<commit_message>
Add machine runtime foundation and workbook sync tooling
</commit_message>
<xml_diff>
--- a/master_data/SAR41-MAS-004_SPS_I-Os.xlsx
+++ b/master_data/SAR41-MAS-004_SPS_I-Os.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://veralto.sharepoint.com/sites/vti/DE-SMD-Support/Switzerland/Shared Documents/11_SAR/01_CH/SAR41-MAS-004_Roche_TTO_LSR_Label und Kontrollsystem_V2/03_Dokumentation/SPS I_Os/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{AB8C5D28-FA20-4A1B-8D10-F83328E299CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F458D271-AFBE-4FF6-9B3F-02F8F5E18652}"/>
+  <xr:revisionPtr revIDLastSave="238" documentId="13_ncr:1_{AB8C5D28-FA20-4A1B-8D10-F83328E299CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9B732FB-4314-4924-87FF-B2D6C5B63653}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{22F4E776-9E13-4485-B5F7-2852C2267A79}"/>
+    <workbookView xWindow="25095" yWindow="0" windowWidth="8595" windowHeight="15135" xr2:uid="{22F4E776-9E13-4485-B5F7-2852C2267A79}"/>
   </bookViews>
   <sheets>
     <sheet name="Raspberry PLC 21 PINOUT" sheetId="2" r:id="rId1"/>
@@ -560,12 +560,6 @@
     <t>Etikettenerfassung Bahnriss</t>
   </si>
   <si>
-    <t>Interrupt Sensor Auswurfkontrolle Bahnriss</t>
-  </si>
-  <si>
-    <t>Auswurfkontrolle Etikette anwesend</t>
-  </si>
-  <si>
     <t>Interrupt Sensor Etikettenerfassung Etikette anwesend</t>
   </si>
   <si>
@@ -579,6 +573,12 @@
   </si>
   <si>
     <t xml:space="preserve">LED Maschinenstatus blau </t>
+  </si>
+  <si>
+    <t>Interrupt Auswurfkontrolle Etikette anwesend</t>
+  </si>
+  <si>
+    <t>Sensor Auswurfkontrolle Bahnriss</t>
   </si>
 </sst>
 </file>
@@ -624,7 +624,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -634,6 +634,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -702,7 +708,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -710,7 +716,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -718,6 +723,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1055,25 +1069,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CE78816-5180-4226-B8C8-C2ABA3FB69C3}">
   <dimension ref="A1:C26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="1" max="2" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:3" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="9"/>
       <c r="C1" s="4"/>
     </row>
-    <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1081,163 +1095,163 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="2"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="10" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
+      <c r="B18" s="14"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="10" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="10" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="10" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1258,27 +1272,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38D5BE34-1B93-443E-912F-AAE2F56CA3D5}">
   <dimension ref="A1:F77"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
     <col min="6" max="6" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="9"/>
       <c r="C1" s="4"/>
     </row>
-    <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1287,191 +1301,191 @@
       </c>
       <c r="F4" s="6"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="10" t="s">
         <v>149</v>
       </c>
       <c r="F5" s="6"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="10" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="10" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="10" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="B11" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="B12" s="11" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="11" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="11" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B18" s="5"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="8"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="10" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="10" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="B23" s="10" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="10" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="11" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:2" ht="21" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>2</v>
       </c>
@@ -1479,174 +1493,174 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="10" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="10" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="10" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="10" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="10" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="10" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="10" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="11" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>64</v>
       </c>
       <c r="B40" s="2"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B41" s="2"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B42" s="2"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B43" s="2"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B44" s="5"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="8"/>
-      <c r="B45" s="9"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="7"/>
+      <c r="B45" s="8"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="10" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="10" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="10" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="10" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="10" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:2" ht="21" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>2</v>
       </c>
@@ -1654,159 +1668,159 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="11" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="2" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="11" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="2" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="10" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="2" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="10" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" s="2" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="10" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" s="2" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="10" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="10" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="2" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="10" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" s="2" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="2" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" s="8"/>
-      <c r="B69" s="9"/>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" s="2" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="7"/>
+      <c r="B69" s="8"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="10" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" s="2" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" s="10" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="2" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="B72" s="12" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" s="10" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="2" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="10" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" s="2" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" s="10" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="2" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="2" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" s="10" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1829,21 +1843,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498EB550-9F97-4177-861B-475832A9E278}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:3" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="9"/>
       <c r="C1" s="4"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1851,127 +1865,127 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="10" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="10" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="10" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="10" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>131</v>
       </c>
@@ -1993,21 +2007,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A13691BF-7D11-40F4-AC6C-FA7A07658944}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:3" ht="24" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="9"/>
       <c r="C1" s="4"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2015,113 +2029,113 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="10" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="10" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="10" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="10" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="10" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="10" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>124</v>
       </c>
       <c r="B12" s="2"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>125</v>
       </c>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>126</v>
       </c>
       <c r="B14" s="2"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>127</v>
       </c>
       <c r="B15" s="2"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>128</v>
       </c>
       <c r="B16" s="2"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>129</v>
       </c>
       <c r="B17" s="2"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>130</v>
       </c>
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>131</v>
       </c>
@@ -2140,15 +2154,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
@@ -2157,6 +2162,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2420,20 +2434,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{374C58C1-F431-4285-AA95-372A85536EF9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E194F7D3-BE2D-4C3A-8879-7C5D41CE2FEC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
     <ds:schemaRef ds:uri="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{374C58C1-F431-4285-AA95-372A85536EF9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Add laser safety reset interlock
</commit_message>
<xml_diff>
--- a/master_data/SAR41-MAS-004_SPS_I-Os.xlsx
+++ b/master_data/SAR41-MAS-004_SPS_I-Os.xlsx
@@ -10,6 +10,7 @@
     <sheet name="ESP32 PLC 58 PINOUT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="IOLOGIK E1211 PINOUT Modul 1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="IOLOGIK E1211 PINOUT Modul 2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IOLOGIK E1213 PINOUT Modul 1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1082,7 +1083,11 @@
           <t>I0.12</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Laser System Ready</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="n"/>
@@ -1184,8 +1189,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30" ht="21" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
@@ -1441,8 +1444,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56" ht="21" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
@@ -1698,8 +1699,8 @@
   <mergeCells count="4">
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -2164,294 +2165,53 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC1303956E7B004BAA4FB741FFD4FB75" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8a32518fee107c04aa9bd7948c0d3f18">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9c94746f-923d-44d4-92c8-8aca0d670c40" xmlns:ns3="045083a1-3069-4c94-ae09-233755b46388" xmlns:ns4="d728571b-78ef-4dbd-85be-d4d1cda44c95" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e97db55af52189d57b3fce0d0bdbaea8" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="9c94746f-923d-44d4-92c8-8aca0d670c40"/>
-    <xsd:import namespace="045083a1-3069-4c94-ae09-233755b46388"/>
-    <xsd:import namespace="d728571b-78ef-4dbd-85be-d4d1cda44c95"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9c94746f-923d-44d4-92c8-8aca0d670c40" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="11" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="15" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:internalName="MediaServiceKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="Length (seconds)" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="23" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1512ac1f-2332-492c-8cad-e2606caf05d8" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="24" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="25" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="045083a1-3069-4c94-ae09-233755b46388" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d728571b-78ef-4dbd-85be-d4d1cda44c95" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3e60fd20-1b61-4c9c-a058-6e112eef0d0c}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="d728571b-78ef-4dbd-85be-d4d1cda44c95">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9c94746f-923d-44d4-92c8-8aca0d670c40">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d728571b-78ef-4dbd-85be-d4d1cda44c95" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57B891BF-5E5D-495E-8139-A8302E798C2E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEB75571-12FF-49C8-A447-4147E8C00AA4}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{609BEE36-8180-4725-9EBF-9CFDEC07736C}"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28.5703125" customWidth="1" min="1" max="1"/>
+    <col width="39.28515625" customWidth="1" min="2" max="2"/>
+    <col width="16.85546875" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>IOLOGIK E1213 PINOUT Digital I/Os</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PLC Pinout</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DIO3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reset Sicherheitskreis Laser</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remap Moxa IO master to E1213
</commit_message>
<xml_diff>
--- a/master_data/SAR41-MAS-004_SPS_I-Os.xlsx
+++ b/master_data/SAR41-MAS-004_SPS_I-Os.xlsx
@@ -8,9 +8,9 @@
   <sheets>
     <sheet name="Raspberry PLC 21 PINOUT" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ESP32 PLC 58 PINOUT" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="IOLOGIK E1211 PINOUT Modul 1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="IOLOGIK E1211 PINOUT Modul 2" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="IOLOGIK E1213 PINOUT Modul 1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="IOLOGIK E1213 PINOUT Modul 1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="IOLOGIK E1213 PINOUT Modul 2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IOLOGIK E1213 PINOUT Modul 3" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1699,8 +1699,8 @@
   <mergeCells count="4">
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A69:B69"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A69:B69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -1721,21 +1721,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="39.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="28.5703125" customWidth="1" min="1" max="1"/>
+    <col width="39.28515625" customWidth="1" min="2" max="2"/>
     <col width="16.85546875" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>IOLOGIK E1211 PINOUT Digital I/Os</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="n"/>
+          <t>IOLOGIK E1213 PINOUT Digital I/Os</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1750,207 +1749,103 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>DO0</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor X-Achse (IN0)</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Schutzblech Laser</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>DO1</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor X-Achse</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Start Motor Kamera Materialkontrolle (IN0)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>DO2</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 2 Motor X-Achse</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Kamera Materialkontrolle</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>DO3</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor Z-Achse (IN0)</t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Start Motor Etikettenanschlag rechts (IN0)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>DO4</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor Z-Achse</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIO0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Etikettenanschlag rechts</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>DO5</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 2 Motor Z-Achse</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DIO1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Start Motor Etikettenanschlag links (IN0)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>DO6</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor Etikettenantrieb</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DIO2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Etikettenanschlag links</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>DO7</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 2 Motor Etikettenantrieb</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>DO8</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor Schutzblech Laser</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>DO9</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor Kamera Materialkontrolle (IN0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>DO10</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor Kamera Materialkontrolle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>DO11</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor Etikettenanschlag rechts (IN0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>DO12</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor Etikettenanschlag rechts</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>DO13</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor Etikettenanschlag links (IN0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>DO14</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Reserve 1 Motor Etikettenanschlag links</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>DO15</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DIO3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Reset Sicherheitskreis Laser</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;"Default"&amp;10 &amp;KD89B2B_x000d_# Confidential - Company Proprietary</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1960,21 +1855,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="39.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="28.5703125" customWidth="1" min="1" max="1"/>
+    <col width="39.28515625" customWidth="1" min="2" max="2"/>
     <col width="16.85546875" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>IOLOGIK E1211 PINOUT Digital I/Os</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="n"/>
+          <t>IOLOGIK E1213 PINOUT Digital I/Os</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1989,179 +1883,103 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>DO0</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor Etikettenanwesenheit (IN0)</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Start Motor X-Achse (IN0)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>DO1</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Start Motor Auswurfkontrolle (IN0)</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor X-Achse</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>DO2</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reserve 1 Motor Etikettenanwesenheit </t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Reserve 2 Motor X-Achse</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>DO3</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reserve 1 Motor Auswurfkontrolle </t>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Start Motor Z-Achse (IN0)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>DO4</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>LED Maschinenstatus rot</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIO0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Z-Achse</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>DO5</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>LED Maschinenstatus grün</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DIO1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Reserve 2 Motor Z-Achse</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>DO6</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LED Maschinenstatus blau </t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DIO2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Etikettenantrieb</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>DO7</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Teach Sensor Etikettenerfassung</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>DO8</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>DO9</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>DO10</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>DO11</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>DO12</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>DO13</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>DO14</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>DO15</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DIO3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Reserve 2 Motor Etikettenantrieb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;"Default"&amp;10 &amp;KD89B2B_x000d_# Confidential - Company Proprietary</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2171,7 +1989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28.5703125" customWidth="1" min="1" max="1"/>
@@ -2186,7 +2004,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2202,12 +2019,96 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>DO0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Start Motor Etikettenanwesenheit (IN0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DO1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Start Motor Auswurfkontrolle (IN0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DO2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Etikettenanwesenheit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DO3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Reserve 1 Motor Auswurfkontrolle</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIO0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LED Maschinenstatus rot</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DIO1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LED Maschinenstatus gruen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DIO2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LED Maschinenstatus blau</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>DIO3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Reset Sicherheitskreis Laser</t>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Teach Sensor Etikettenerfassung</t>
         </is>
       </c>
     </row>

</xml_diff>